<commit_message>
update to events list
</commit_message>
<xml_diff>
--- a/Events.xlsx
+++ b/Events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mdigital-my.sharepoint.com/personal/m269810_one_merckgroup_com/Documents/Documents/LegacyHomeDriveDocuments/EFSPI/calendar/calendar/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="8_{C02827F6-0260-4401-9323-2DCC0C6C1E05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5D2FDF1-384F-4FC1-8789-51D2C95E1AEF}"/>
+  <xr:revisionPtr revIDLastSave="94" documentId="8_{C02827F6-0260-4401-9323-2DCC0C6C1E05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F6D413B-04CC-41D2-8BD3-DCE959428953}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3AD4CD51-029A-4D3E-BCE9-D3BABE131D5C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3AD4CD51-029A-4D3E-BCE9-D3BABE131D5C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="56">
   <si>
     <t>Title</t>
   </si>
@@ -86,9 +86,6 @@
     <t>APF Workshop</t>
   </si>
   <si>
-    <t>Frankfurt</t>
-  </si>
-  <si>
     <t>Making Estimands Work - Practical Approaches with Implementation in Data Standards</t>
   </si>
   <si>
@@ -156,6 +153,60 @@
   </si>
   <si>
     <t>Digital Innovation in Healthcare (3): AI, Data and Emerging Technologies</t>
+  </si>
+  <si>
+    <t>Exploratory Subgroup Analyses in Clinical Trials</t>
+  </si>
+  <si>
+    <t>BBS</t>
+  </si>
+  <si>
+    <t>14:00  - 17:30</t>
+  </si>
+  <si>
+    <t>https://baselbiometrics.github.io/home/docs/upcoming/20261201/agenda.pdf</t>
+  </si>
+  <si>
+    <t>https://forms.cloud.microsoft/pages/responsepage.aspx?id=Turct1DRoUuLKsiyenVSXCAIESSLFaJAphQ9wzm6v9tUQTFZUUYwU1hINTVRQkZLTEVYRUdBMkJCMi4u&amp;route=shorturl</t>
+  </si>
+  <si>
+    <t>Quantitative Drug Development in the Age of AI</t>
+  </si>
+  <si>
+    <t>14:00 - 18:00</t>
+  </si>
+  <si>
+    <t>CHF 50</t>
+  </si>
+  <si>
+    <t>https://baselbiometrics.github.io/home/docs/upcoming/20261110/agenda.pdf</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSdEyA85vPNxDv3ar6rOH6QfVFViEfapziahRXYNal53c-2NLw/viewform</t>
+  </si>
+  <si>
+    <t>Bayesian Drug Development through the lens of ICH M15</t>
+  </si>
+  <si>
+    <t>BBS / EFSPI</t>
+  </si>
+  <si>
+    <t>EUR 60</t>
+  </si>
+  <si>
+    <t>https://baselbiometrics.github.io/home/docs/upcoming/20261210/agenda.pdf</t>
+  </si>
+  <si>
+    <t>https://www.efspi.org/product/bayesian-drug-development-through-the-lens-of-ich-m15/</t>
+  </si>
+  <si>
+    <t>https://www.biometrische-gesellschaft.de/pdf/APF_Conference_Agenda%202026%20Fulda_VL.pdf</t>
+  </si>
+  <si>
+    <t>https://forms.cloud.microsoft/Pages/ResponsePage.aspx?id=czWRwTbFE0y866Zxpm5yPJn785MmOGpFoCLmVLEcXzxUOUpNNkNXMkRVVEhITFJQWkZXMVo2NUE1Sy4u</t>
+  </si>
+  <si>
+    <t>Fulda</t>
   </si>
 </sst>
 </file>
@@ -545,17 +596,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7FF786E-2CBC-43F4-BB59-B074A7E1A64E}">
-  <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -581,7 +632,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -595,7 +646,7 @@
         <v>46253</v>
       </c>
       <c r="F2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>11</v>
@@ -604,7 +655,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -612,149 +663,230 @@
         <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="D3" s="1">
         <v>46353</v>
       </c>
       <c r="F3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+        <v>23</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
         <v>16</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
       </c>
       <c r="D4" s="1">
         <v>46294</v>
       </c>
       <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>21</v>
-      </c>
       <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
         <v>17</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
       </c>
       <c r="D5" s="1">
         <v>46315</v>
       </c>
       <c r="F5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H5" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
         <v>27</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>28</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
       </c>
       <c r="D6" s="1">
         <v>46317</v>
       </c>
       <c r="F6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D7" s="1">
         <v>46279</v>
       </c>
       <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
         <v>32</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D8" s="1">
         <v>46345</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F8" t="s">
+        <v>32</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D9" s="1">
         <v>46370</v>
       </c>
       <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" t="s">
         <v>32</v>
       </c>
-      <c r="F9" t="s">
+      <c r="H9" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D10" s="1"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="1">
+        <v>46357</v>
+      </c>
+      <c r="E10" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="1">
+        <v>46336</v>
+      </c>
+      <c r="E11" t="s">
+        <v>44</v>
+      </c>
+      <c r="F11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="1">
+        <v>46366</v>
+      </c>
+      <c r="E12" t="s">
+        <v>44</v>
+      </c>
+      <c r="F12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>52</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -767,6 +899,12 @@
     <hyperlink ref="H7" r:id="rId6" xr:uid="{74B81336-B77E-4FE3-B292-3EC638C8D38C}"/>
     <hyperlink ref="H8" r:id="rId7" xr:uid="{89A74A77-045F-48B7-87C5-97737ACA562C}"/>
     <hyperlink ref="H9" r:id="rId8" xr:uid="{9D96AAE2-3517-4194-AB05-F87AF4D3141C}"/>
+    <hyperlink ref="G11" r:id="rId9" xr:uid="{30C01C0E-2F3B-4108-AB9E-934A8373194E}"/>
+    <hyperlink ref="H11" r:id="rId10" xr:uid="{E952C1F2-2236-4CBF-B4D0-A77DF33A4EC5}"/>
+    <hyperlink ref="G12" r:id="rId11" xr:uid="{F13A072F-DCBD-497E-868C-A8079EC93AC7}"/>
+    <hyperlink ref="H12" r:id="rId12" xr:uid="{246D4972-EB91-432A-B00A-D83EB39DFF8F}"/>
+    <hyperlink ref="G3" r:id="rId13" xr:uid="{1F8D6EFA-FA35-4959-B011-7CD94431D671}"/>
+    <hyperlink ref="H3" r:id="rId14" xr:uid="{52C5079B-AEFC-4D60-AFAA-D75F5C93EE7A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>